<commit_message>
Incorporación de noticias manuales relevantes
</commit_message>
<xml_diff>
--- a/Output/INEGI_Data/series_inegi_consolidadas.xlsx
+++ b/Output/INEGI_Data/series_inegi_consolidadas.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="serie_7" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="serie_8" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="serie_9" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="serie_10" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -811,6 +812,44 @@
       </c>
       <c r="H10" t="n">
         <v>-5.699800062055</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>serie_10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Indicador 496434</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Por determinar</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>mensual</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>87</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2016-03-01</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2023-05-01</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>4.003280784883</v>
       </c>
     </row>
   </sheetData>
@@ -2552,6 +2591,1740 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F88"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Cambio mensual (%)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Cambio anual (%)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Promedio 3M</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Promedio 12M</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>42430</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-1.448824562991</v>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>42461</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-0.768885891768</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-46.93036607685009</v>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>42491</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-0.048937722246</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-93.63524252818958</v>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>-0.755549392335</v>
+      </c>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>42522</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.449831821403</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-1019.192395473142</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>-0.1226639308703334</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>42552</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.6751241293270001</v>
+      </c>
+      <c r="C6" t="n">
+        <v>50.08367509913507</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="n">
+        <v>0.358672742828</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>42583</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.393998734289</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-41.64054917104517</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>0.5063182283396667</v>
+      </c>
+      <c r="F7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>42614</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.02322093139</v>
+      </c>
+      <c r="C8" t="n">
+        <v>-94.10634365820898</v>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="n">
+        <v>0.3641145983353333</v>
+      </c>
+      <c r="F8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>42644</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-0.283816382554</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-1322.243749775792</v>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>0.04446776104166666</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>42675</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-0.53012296872</v>
+      </c>
+      <c r="C10" t="n">
+        <v>86.78378039686865</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>-0.263572806628</v>
+      </c>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>42705</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-0.632579318297</v>
+      </c>
+      <c r="C11" t="n">
+        <v>19.3269025532669</v>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="n">
+        <v>-0.4821728898570001</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>42736</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.888580628355</v>
+      </c>
+      <c r="C12" t="n">
+        <v>-240.4694403774051</v>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="n">
+        <v>-0.09137388622066667</v>
+      </c>
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>42767</v>
+      </c>
+      <c r="B13" t="n">
+        <v>-0.278073048778</v>
+      </c>
+      <c r="C13" t="n">
+        <v>-131.294070555284</v>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="n">
+        <v>-0.007357246240000004</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-0.1300403042158333</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>42795</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.764684892303</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-374.9942490519774</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-152.7796747678242</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.4583974906266666</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.05441881705866666</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>42826</v>
+      </c>
+      <c r="B15" t="n">
+        <v>-0.339296514462</v>
+      </c>
+      <c r="C15" t="n">
+        <v>-144.3707621109319</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-55.87166859287649</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.04910510968766666</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.09021793183416667</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>42856</v>
+      </c>
+      <c r="B16" t="n">
+        <v>-0.349949382082</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3.139692618679435</v>
+      </c>
+      <c r="D16" t="n">
+        <v>615.0912752393244</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.02514633191966666</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.06513362684783332</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>42887</v>
+      </c>
+      <c r="B17" t="n">
+        <v>-0.369311279646</v>
+      </c>
+      <c r="C17" t="n">
+        <v>5.532770896410133</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-182.0998564517155</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-0.3528523920633334</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-0.003128298239583332</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>42917</v>
+      </c>
+      <c r="B18" t="n">
+        <v>-0.885732952117</v>
+      </c>
+      <c r="C18" t="n">
+        <v>139.8337123539826</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-231.1955703612528</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-0.5349978712816666</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-0.13319972169325</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>42948</v>
+      </c>
+      <c r="B19" t="n">
+        <v>-1.107719444594</v>
+      </c>
+      <c r="C19" t="n">
+        <v>25.06246289543905</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-381.1479703337022</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-0.7875878921189999</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-0.2583429032668333</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>42979</v>
+      </c>
+      <c r="B20" t="n">
+        <v>-0.909515947653</v>
+      </c>
+      <c r="C20" t="n">
+        <v>-17.89293289995872</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-4016.793570324571</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-0.967656114788</v>
+      </c>
+      <c r="F20" t="n">
+        <v>-0.3360709765204167</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>43009</v>
+      </c>
+      <c r="B21" t="n">
+        <v>-1.326872855797</v>
+      </c>
+      <c r="C21" t="n">
+        <v>45.88780540033264</v>
+      </c>
+      <c r="D21" t="n">
+        <v>367.5110167555405</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-1.114702749348</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-0.4229923492906666</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>43040</v>
+      </c>
+      <c r="B22" t="n">
+        <v>-0.900459286152</v>
+      </c>
+      <c r="C22" t="n">
+        <v>-32.136731698296</v>
+      </c>
+      <c r="D22" t="n">
+        <v>69.8585685366906</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-1.045616029867333</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-0.4538537090766666</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>43070</v>
+      </c>
+      <c r="B23" t="n">
+        <v>-0.938201593501</v>
+      </c>
+      <c r="C23" t="n">
+        <v>4.191450732912871</v>
+      </c>
+      <c r="D23" t="n">
+        <v>48.31366855729362</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-1.055177911816666</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-0.4793222320103334</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>43101</v>
+      </c>
+      <c r="B24" t="n">
+        <v>8.355475096198999</v>
+      </c>
+      <c r="C24" t="n">
+        <v>-990.584193640052</v>
+      </c>
+      <c r="D24" t="n">
+        <v>840.3170437855724</v>
+      </c>
+      <c r="E24" t="n">
+        <v>2.172271405515333</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.1429189736433333</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>43132</v>
+      </c>
+      <c r="B25" t="n">
+        <v>9.945198478687001</v>
+      </c>
+      <c r="C25" t="n">
+        <v>19.02612794826215</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-3676.469752243686</v>
+      </c>
+      <c r="E25" t="n">
+        <v>5.787490660461667</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.99485826759875</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>43160</v>
+      </c>
+      <c r="B26" t="n">
+        <v>7.344075648471</v>
+      </c>
+      <c r="C26" t="n">
+        <v>-26.15455926586404</v>
+      </c>
+      <c r="D26" t="n">
+        <v>860.4054849773298</v>
+      </c>
+      <c r="E26" t="n">
+        <v>8.548249741118999</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1.54314083061275</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>43191</v>
+      </c>
+      <c r="B27" t="n">
+        <v>9.144864342119</v>
+      </c>
+      <c r="C27" t="n">
+        <v>24.52029063756873</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-2795.242642447832</v>
+      </c>
+      <c r="E27" t="n">
+        <v>8.811379489759</v>
+      </c>
+      <c r="F27" t="n">
+        <v>2.333487568661166</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>43221</v>
+      </c>
+      <c r="B28" t="n">
+        <v>8.124176946807999</v>
+      </c>
+      <c r="C28" t="n">
+        <v>-11.16131805925173</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-2421.529159009729</v>
+      </c>
+      <c r="E28" t="n">
+        <v>8.204372312465999</v>
+      </c>
+      <c r="F28" t="n">
+        <v>3.039664762735333</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>43252</v>
+      </c>
+      <c r="B29" t="n">
+        <v>8.230148605548999</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1.304398703214305</v>
+      </c>
+      <c r="D29" t="n">
+        <v>-2328.512655621549</v>
+      </c>
+      <c r="E29" t="n">
+        <v>8.499729964825333</v>
+      </c>
+      <c r="F29" t="n">
+        <v>3.756286419834916</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>43282</v>
+      </c>
+      <c r="B30" t="n">
+        <v>9.099910788624999</v>
+      </c>
+      <c r="C30" t="n">
+        <v>10.56800095310044</v>
+      </c>
+      <c r="D30" t="n">
+        <v>-1127.387630422375</v>
+      </c>
+      <c r="E30" t="n">
+        <v>8.484745446993999</v>
+      </c>
+      <c r="F30" t="n">
+        <v>4.588423398230083</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>43313</v>
+      </c>
+      <c r="B31" t="n">
+        <v>9.401508336825</v>
+      </c>
+      <c r="C31" t="n">
+        <v>3.314291262909963</v>
+      </c>
+      <c r="D31" t="n">
+        <v>-948.7264878040331</v>
+      </c>
+      <c r="E31" t="n">
+        <v>8.910522576999666</v>
+      </c>
+      <c r="F31" t="n">
+        <v>5.464192380015</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>43344</v>
+      </c>
+      <c r="B32" t="n">
+        <v>9.599001541812999</v>
+      </c>
+      <c r="C32" t="n">
+        <v>2.100654468543461</v>
+      </c>
+      <c r="D32" t="n">
+        <v>-1155.396726861487</v>
+      </c>
+      <c r="E32" t="n">
+        <v>9.366806889087668</v>
+      </c>
+      <c r="F32" t="n">
+        <v>6.339902170803833</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>43374</v>
+      </c>
+      <c r="B33" t="n">
+        <v>9.820476907264</v>
+      </c>
+      <c r="C33" t="n">
+        <v>2.307275027368827</v>
+      </c>
+      <c r="D33" t="n">
+        <v>-840.1219238421476</v>
+      </c>
+      <c r="E33" t="n">
+        <v>9.606995595300665</v>
+      </c>
+      <c r="F33" t="n">
+        <v>7.26884798439225</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>43405</v>
+      </c>
+      <c r="B34" t="n">
+        <v>9.544676142790999</v>
+      </c>
+      <c r="C34" t="n">
+        <v>-2.808425365462619</v>
+      </c>
+      <c r="D34" t="n">
+        <v>-1159.978645295444</v>
+      </c>
+      <c r="E34" t="n">
+        <v>9.654718197289332</v>
+      </c>
+      <c r="F34" t="n">
+        <v>8.139275936804166</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>43435</v>
+      </c>
+      <c r="B35" t="n">
+        <v>9.158141988888</v>
+      </c>
+      <c r="C35" t="n">
+        <v>-4.049735665415377</v>
+      </c>
+      <c r="D35" t="n">
+        <v>-1076.1379699552</v>
+      </c>
+      <c r="E35" t="n">
+        <v>9.507765012981</v>
+      </c>
+      <c r="F35" t="n">
+        <v>8.980637902003251</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>43466</v>
+      </c>
+      <c r="B36" t="n">
+        <v>-3.617943501178</v>
+      </c>
+      <c r="C36" t="n">
+        <v>-139.5052130177477</v>
+      </c>
+      <c r="D36" t="n">
+        <v>-143.3002726897462</v>
+      </c>
+      <c r="E36" t="n">
+        <v>5.028291543500333</v>
+      </c>
+      <c r="F36" t="n">
+        <v>7.982853018888499</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>43497</v>
+      </c>
+      <c r="B37" t="n">
+        <v>-3.924045777183</v>
+      </c>
+      <c r="C37" t="n">
+        <v>8.460670430738727</v>
+      </c>
+      <c r="D37" t="n">
+        <v>-139.4566864159866</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.5387175701756665</v>
+      </c>
+      <c r="F37" t="n">
+        <v>6.827082664232666</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>43525</v>
+      </c>
+      <c r="B38" t="n">
+        <v>-2.679617001751</v>
+      </c>
+      <c r="C38" t="n">
+        <v>-31.71290158407256</v>
+      </c>
+      <c r="D38" t="n">
+        <v>-136.4867837698388</v>
+      </c>
+      <c r="E38" t="n">
+        <v>-3.407202093370667</v>
+      </c>
+      <c r="F38" t="n">
+        <v>5.991774943380833</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>43556</v>
+      </c>
+      <c r="B39" t="n">
+        <v>-3.290187563271</v>
+      </c>
+      <c r="C39" t="n">
+        <v>22.78573994421671</v>
+      </c>
+      <c r="D39" t="n">
+        <v>-135.9785278401256</v>
+      </c>
+      <c r="E39" t="n">
+        <v>-3.297950114068334</v>
+      </c>
+      <c r="F39" t="n">
+        <v>4.955520617931666</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>43586</v>
+      </c>
+      <c r="B40" t="n">
+        <v>-2.382948600215</v>
+      </c>
+      <c r="C40" t="n">
+        <v>-27.57408037109141</v>
+      </c>
+      <c r="D40" t="n">
+        <v>-129.3315694108714</v>
+      </c>
+      <c r="E40" t="n">
+        <v>-2.784251055079</v>
+      </c>
+      <c r="F40" t="n">
+        <v>4.079926822346416</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>43617</v>
+      </c>
+      <c r="B41" t="n">
+        <v>-2.031124039281</v>
+      </c>
+      <c r="C41" t="n">
+        <v>-14.76425303098259</v>
+      </c>
+      <c r="D41" t="n">
+        <v>-124.6790688312913</v>
+      </c>
+      <c r="E41" t="n">
+        <v>-2.568086734255667</v>
+      </c>
+      <c r="F41" t="n">
+        <v>3.224820768610583</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>43647</v>
+      </c>
+      <c r="B42" t="n">
+        <v>-2.220001853112</v>
+      </c>
+      <c r="C42" t="n">
+        <v>9.299176720780732</v>
+      </c>
+      <c r="D42" t="n">
+        <v>-124.3958639230511</v>
+      </c>
+      <c r="E42" t="n">
+        <v>-2.211358164202667</v>
+      </c>
+      <c r="F42" t="n">
+        <v>2.2814947151325</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>43678</v>
+      </c>
+      <c r="B43" t="n">
+        <v>-1.709002257558</v>
+      </c>
+      <c r="C43" t="n">
+        <v>-23.0179805858126</v>
+      </c>
+      <c r="D43" t="n">
+        <v>-118.1779582204269</v>
+      </c>
+      <c r="E43" t="n">
+        <v>-1.986709383317</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1.35561883226725</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>43709</v>
+      </c>
+      <c r="B44" t="n">
+        <v>-1.22676827939</v>
+      </c>
+      <c r="C44" t="n">
+        <v>-28.21728151822725</v>
+      </c>
+      <c r="D44" t="n">
+        <v>-112.7801654583159</v>
+      </c>
+      <c r="E44" t="n">
+        <v>-1.718590796686667</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.4534713471669998</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>43739</v>
+      </c>
+      <c r="B45" t="n">
+        <v>-0.689906306524</v>
+      </c>
+      <c r="C45" t="n">
+        <v>-43.76229658733515</v>
+      </c>
+      <c r="D45" t="n">
+        <v>-107.0251812925062</v>
+      </c>
+      <c r="E45" t="n">
+        <v>-1.208558947824</v>
+      </c>
+      <c r="F45" t="n">
+        <v>-0.4223939206486668</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>43770</v>
+      </c>
+      <c r="B46" t="n">
+        <v>-0.458583596145</v>
+      </c>
+      <c r="C46" t="n">
+        <v>-33.52958339292307</v>
+      </c>
+      <c r="D46" t="n">
+        <v>-104.8046009030004</v>
+      </c>
+      <c r="E46" t="n">
+        <v>-0.791752727353</v>
+      </c>
+      <c r="F46" t="n">
+        <v>-1.255998898893333</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>43800</v>
+      </c>
+      <c r="B47" t="n">
+        <v>-0.021194607826</v>
+      </c>
+      <c r="C47" t="n">
+        <v>-95.37824553600072</v>
+      </c>
+      <c r="D47" t="n">
+        <v>-100.2314291245071</v>
+      </c>
+      <c r="E47" t="n">
+        <v>-0.3898948368316666</v>
+      </c>
+      <c r="F47" t="n">
+        <v>-2.020943615286167</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>43831</v>
+      </c>
+      <c r="B48" t="n">
+        <v>-1.901300408679</v>
+      </c>
+      <c r="C48" t="n">
+        <v>8870.679827095566</v>
+      </c>
+      <c r="D48" t="n">
+        <v>-47.44803482807463</v>
+      </c>
+      <c r="E48" t="n">
+        <v>-0.7936928708833334</v>
+      </c>
+      <c r="F48" t="n">
+        <v>-1.877890024244583</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>43862</v>
+      </c>
+      <c r="B49" t="n">
+        <v>-0.223034873783</v>
+      </c>
+      <c r="C49" t="n">
+        <v>-88.26935118906528</v>
+      </c>
+      <c r="D49" t="n">
+        <v>-94.31620102191793</v>
+      </c>
+      <c r="E49" t="n">
+        <v>-0.715176630096</v>
+      </c>
+      <c r="F49" t="n">
+        <v>-1.56947244896125</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>43891</v>
+      </c>
+      <c r="B50" t="n">
+        <v>-0.416026914053</v>
+      </c>
+      <c r="C50" t="n">
+        <v>86.52998385255665</v>
+      </c>
+      <c r="D50" t="n">
+        <v>-84.47438892270252</v>
+      </c>
+      <c r="E50" t="n">
+        <v>-0.8467873988383333</v>
+      </c>
+      <c r="F50" t="n">
+        <v>-1.380839941653083</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>43922</v>
+      </c>
+      <c r="B51" t="n">
+        <v>-0.949380716778</v>
+      </c>
+      <c r="C51" t="n">
+        <v>128.2017544319388</v>
+      </c>
+      <c r="D51" t="n">
+        <v>-71.14508828079832</v>
+      </c>
+      <c r="E51" t="n">
+        <v>-0.5294808348713334</v>
+      </c>
+      <c r="F51" t="n">
+        <v>-1.185772704445333</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
+        <v>43952</v>
+      </c>
+      <c r="B52" t="n">
+        <v>-3.818414606958</v>
+      </c>
+      <c r="C52" t="n">
+        <v>302.2005650079878</v>
+      </c>
+      <c r="D52" t="n">
+        <v>60.23906712102334</v>
+      </c>
+      <c r="E52" t="n">
+        <v>-1.727940745929667</v>
+      </c>
+      <c r="F52" t="n">
+        <v>-1.305394871673917</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>43983</v>
+      </c>
+      <c r="B53" t="n">
+        <v>-5.798169748458</v>
+      </c>
+      <c r="C53" t="n">
+        <v>51.84756882849877</v>
+      </c>
+      <c r="D53" t="n">
+        <v>185.4660590059532</v>
+      </c>
+      <c r="E53" t="n">
+        <v>-3.521988357398</v>
+      </c>
+      <c r="F53" t="n">
+        <v>-1.619315347438667</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>44013</v>
+      </c>
+      <c r="B54" t="n">
+        <v>-6.149943046701</v>
+      </c>
+      <c r="C54" t="n">
+        <v>6.066971363447093</v>
+      </c>
+      <c r="D54" t="n">
+        <v>177.0242303212497</v>
+      </c>
+      <c r="E54" t="n">
+        <v>-5.255509134038999</v>
+      </c>
+      <c r="F54" t="n">
+        <v>-1.946810446904417</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>44044</v>
+      </c>
+      <c r="B55" t="n">
+        <v>-5.645857142254</v>
+      </c>
+      <c r="C55" t="n">
+        <v>-8.196594677692271</v>
+      </c>
+      <c r="D55" t="n">
+        <v>230.3598410877109</v>
+      </c>
+      <c r="E55" t="n">
+        <v>-5.864656645804334</v>
+      </c>
+      <c r="F55" t="n">
+        <v>-2.27488168729575</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n">
+        <v>44075</v>
+      </c>
+      <c r="B56" t="n">
+        <v>-5.896328046279</v>
+      </c>
+      <c r="C56" t="n">
+        <v>4.436366307437312</v>
+      </c>
+      <c r="D56" t="n">
+        <v>380.6391023748102</v>
+      </c>
+      <c r="E56" t="n">
+        <v>-5.897376078411334</v>
+      </c>
+      <c r="F56" t="n">
+        <v>-2.664011667869833</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
+        <v>44105</v>
+      </c>
+      <c r="B57" t="n">
+        <v>-6.11741986257</v>
+      </c>
+      <c r="C57" t="n">
+        <v>3.749652572850404</v>
+      </c>
+      <c r="D57" t="n">
+        <v>786.7029920905923</v>
+      </c>
+      <c r="E57" t="n">
+        <v>-5.886535017034333</v>
+      </c>
+      <c r="F57" t="n">
+        <v>-3.116304464207</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n">
+        <v>44136</v>
+      </c>
+      <c r="B58" t="n">
+        <v>-6.658265167002</v>
+      </c>
+      <c r="C58" t="n">
+        <v>8.84106889149805</v>
+      </c>
+      <c r="D58" t="n">
+        <v>1351.919611380237</v>
+      </c>
+      <c r="E58" t="n">
+        <v>-6.224004358617001</v>
+      </c>
+      <c r="F58" t="n">
+        <v>-3.63294459511175</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>44166</v>
+      </c>
+      <c r="B59" t="n">
+        <v>-6.975875130765</v>
+      </c>
+      <c r="C59" t="n">
+        <v>4.770160932265921</v>
+      </c>
+      <c r="D59" t="n">
+        <v>32813.44283430196</v>
+      </c>
+      <c r="E59" t="n">
+        <v>-6.583853386779</v>
+      </c>
+      <c r="F59" t="n">
+        <v>-4.212501305356667</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
+        <v>44197</v>
+      </c>
+      <c r="B60" t="n">
+        <v>-22.806206248155</v>
+      </c>
+      <c r="C60" t="n">
+        <v>226.9296800852281</v>
+      </c>
+      <c r="D60" t="n">
+        <v>1099.505672225699</v>
+      </c>
+      <c r="E60" t="n">
+        <v>-12.146782181974</v>
+      </c>
+      <c r="F60" t="n">
+        <v>-5.954576791979666</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>44228</v>
+      </c>
+      <c r="B61" t="n">
+        <v>-26.017367294611</v>
+      </c>
+      <c r="C61" t="n">
+        <v>14.08020699065535</v>
+      </c>
+      <c r="D61" t="n">
+        <v>11565.15659785312</v>
+      </c>
+      <c r="E61" t="n">
+        <v>-18.59981622451033</v>
+      </c>
+      <c r="F61" t="n">
+        <v>-8.104104493715333</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>44256</v>
+      </c>
+      <c r="B62" t="n">
+        <v>-24.992398194303</v>
+      </c>
+      <c r="C62" t="n">
+        <v>-3.939557329923626</v>
+      </c>
+      <c r="D62" t="n">
+        <v>5907.399365301419</v>
+      </c>
+      <c r="E62" t="n">
+        <v>-24.60532391235633</v>
+      </c>
+      <c r="F62" t="n">
+        <v>-10.15213543373617</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>44287</v>
+      </c>
+      <c r="B63" t="n">
+        <v>-24.898106938126</v>
+      </c>
+      <c r="C63" t="n">
+        <v>-0.3772797450006027</v>
+      </c>
+      <c r="D63" t="n">
+        <v>2522.562950575295</v>
+      </c>
+      <c r="E63" t="n">
+        <v>-25.30262414234667</v>
+      </c>
+      <c r="F63" t="n">
+        <v>-12.1478626188485</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>44317</v>
+      </c>
+      <c r="B64" t="n">
+        <v>-22.696768174445</v>
+      </c>
+      <c r="C64" t="n">
+        <v>-8.84139010709336</v>
+      </c>
+      <c r="D64" t="n">
+        <v>494.402926625266</v>
+      </c>
+      <c r="E64" t="n">
+        <v>-24.195757768958</v>
+      </c>
+      <c r="F64" t="n">
+        <v>-13.72105874947242</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>44348</v>
+      </c>
+      <c r="B65" t="n">
+        <v>-21.455578469437</v>
+      </c>
+      <c r="C65" t="n">
+        <v>-5.468574624670552</v>
+      </c>
+      <c r="D65" t="n">
+        <v>270.0405369322453</v>
+      </c>
+      <c r="E65" t="n">
+        <v>-23.01681786066933</v>
+      </c>
+      <c r="F65" t="n">
+        <v>-15.025842809554</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>44378</v>
+      </c>
+      <c r="B66" t="n">
+        <v>-20.978738140006</v>
+      </c>
+      <c r="C66" t="n">
+        <v>-2.222453848588835</v>
+      </c>
+      <c r="D66" t="n">
+        <v>241.1208523509755</v>
+      </c>
+      <c r="E66" t="n">
+        <v>-21.71036159462933</v>
+      </c>
+      <c r="F66" t="n">
+        <v>-16.26157573399608</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>44409</v>
+      </c>
+      <c r="B67" t="n">
+        <v>-22.006960975817</v>
+      </c>
+      <c r="C67" t="n">
+        <v>4.901261596140527</v>
+      </c>
+      <c r="D67" t="n">
+        <v>289.7895469425771</v>
+      </c>
+      <c r="E67" t="n">
+        <v>-21.48042586175333</v>
+      </c>
+      <c r="F67" t="n">
+        <v>-17.62500105345967</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>44440</v>
+      </c>
+      <c r="B68" t="n">
+        <v>-22.640765394806</v>
+      </c>
+      <c r="C68" t="n">
+        <v>2.880017916537736</v>
+      </c>
+      <c r="D68" t="n">
+        <v>283.9807625543142</v>
+      </c>
+      <c r="E68" t="n">
+        <v>-21.87548817020967</v>
+      </c>
+      <c r="F68" t="n">
+        <v>-19.02037083250358</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>44470</v>
+      </c>
+      <c r="B69" t="n">
+        <v>-22.897838669526</v>
+      </c>
+      <c r="C69" t="n">
+        <v>1.135444276009223</v>
+      </c>
+      <c r="D69" t="n">
+        <v>274.305494537469</v>
+      </c>
+      <c r="E69" t="n">
+        <v>-22.51518834671633</v>
+      </c>
+      <c r="F69" t="n">
+        <v>-20.41873906641658</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>44501</v>
+      </c>
+      <c r="B70" t="n">
+        <v>-22.981218459755</v>
+      </c>
+      <c r="C70" t="n">
+        <v>0.3641382552841854</v>
+      </c>
+      <c r="D70" t="n">
+        <v>245.1532476304589</v>
+      </c>
+      <c r="E70" t="n">
+        <v>-22.83994084136233</v>
+      </c>
+      <c r="F70" t="n">
+        <v>-21.778985174146</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>44531</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-22.66073741673</v>
+      </c>
+      <c r="C71" t="n">
+        <v>-1.394534600444397</v>
+      </c>
+      <c r="D71" t="n">
+        <v>224.8443670786427</v>
+      </c>
+      <c r="E71" t="n">
+        <v>-22.84659818200366</v>
+      </c>
+      <c r="F71" t="n">
+        <v>-23.08605703130975</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>44562</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-0.870821446539</v>
+      </c>
+      <c r="C72" t="n">
+        <v>-96.15713544301481</v>
+      </c>
+      <c r="D72" t="n">
+        <v>-96.18164706105186</v>
+      </c>
+      <c r="E72" t="n">
+        <v>-15.50425910767466</v>
+      </c>
+      <c r="F72" t="n">
+        <v>-21.25810829784175</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>44593</v>
+      </c>
+      <c r="B73" t="n">
+        <v>0.396430547642</v>
+      </c>
+      <c r="C73" t="n">
+        <v>-145.5237464829991</v>
+      </c>
+      <c r="D73" t="n">
+        <v>-101.5237150752148</v>
+      </c>
+      <c r="E73" t="n">
+        <v>-7.711709438542333</v>
+      </c>
+      <c r="F73" t="n">
+        <v>-19.056958477654</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>44621</v>
+      </c>
+      <c r="B74" t="n">
+        <v>1.110521314816</v>
+      </c>
+      <c r="C74" t="n">
+        <v>180.1301063758754</v>
+      </c>
+      <c r="D74" t="n">
+        <v>-104.443436384865</v>
+      </c>
+      <c r="E74" t="n">
+        <v>0.212043471973</v>
+      </c>
+      <c r="F74" t="n">
+        <v>-16.88171518522742</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>44652</v>
+      </c>
+      <c r="B75" t="n">
+        <v>1.51389256899</v>
+      </c>
+      <c r="C75" t="n">
+        <v>36.32269356674471</v>
+      </c>
+      <c r="D75" t="n">
+        <v>-106.0803521036846</v>
+      </c>
+      <c r="E75" t="n">
+        <v>1.006948143816</v>
+      </c>
+      <c r="F75" t="n">
+        <v>-14.68071522630108</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>44682</v>
+      </c>
+      <c r="B76" t="n">
+        <v>2.576129809667</v>
+      </c>
+      <c r="C76" t="n">
+        <v>70.16595909349606</v>
+      </c>
+      <c r="D76" t="n">
+        <v>-111.3502054119209</v>
+      </c>
+      <c r="E76" t="n">
+        <v>1.733514564491</v>
+      </c>
+      <c r="F76" t="n">
+        <v>-12.57464039429175</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>44713</v>
+      </c>
+      <c r="B77" t="n">
+        <v>3.178993268758</v>
+      </c>
+      <c r="C77" t="n">
+        <v>23.40190532436439</v>
+      </c>
+      <c r="D77" t="n">
+        <v>-114.8166281011085</v>
+      </c>
+      <c r="E77" t="n">
+        <v>2.423005215805</v>
+      </c>
+      <c r="F77" t="n">
+        <v>-10.52175941610883</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>44743</v>
+      </c>
+      <c r="B78" t="n">
+        <v>3.261853705567</v>
+      </c>
+      <c r="C78" t="n">
+        <v>2.606499284642161</v>
+      </c>
+      <c r="D78" t="n">
+        <v>-115.5483789530063</v>
+      </c>
+      <c r="E78" t="n">
+        <v>3.005658927997333</v>
+      </c>
+      <c r="F78" t="n">
+        <v>-8.501710095644418</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
+        <v>44774</v>
+      </c>
+      <c r="B79" t="n">
+        <v>3.776745118381</v>
+      </c>
+      <c r="C79" t="n">
+        <v>15.7852392930816</v>
+      </c>
+      <c r="D79" t="n">
+        <v>-117.1615932001297</v>
+      </c>
+      <c r="E79" t="n">
+        <v>3.405864030902</v>
+      </c>
+      <c r="F79" t="n">
+        <v>-6.353067921127916</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="n">
+        <v>44805</v>
+      </c>
+      <c r="B80" t="n">
+        <v>4.170931013924</v>
+      </c>
+      <c r="C80" t="n">
+        <v>10.43718554436044</v>
+      </c>
+      <c r="D80" t="n">
+        <v>-118.4222173640863</v>
+      </c>
+      <c r="E80" t="n">
+        <v>3.736509945957334</v>
+      </c>
+      <c r="F80" t="n">
+        <v>-4.118759887067083</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>44835</v>
+      </c>
+      <c r="B81" t="n">
+        <v>4.314390651319</v>
+      </c>
+      <c r="C81" t="n">
+        <v>3.439511152691876</v>
+      </c>
+      <c r="D81" t="n">
+        <v>-118.8419121716535</v>
+      </c>
+      <c r="E81" t="n">
+        <v>4.087355594541333</v>
+      </c>
+      <c r="F81" t="n">
+        <v>-1.85107411033</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="n">
+        <v>44866</v>
+      </c>
+      <c r="B82" t="n">
+        <v>4.500012751464</v>
+      </c>
+      <c r="C82" t="n">
+        <v>4.302394362185336</v>
+      </c>
+      <c r="D82" t="n">
+        <v>-119.581262670404</v>
+      </c>
+      <c r="E82" t="n">
+        <v>4.328444805569</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0.4390284906049167</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="n">
+        <v>44896</v>
+      </c>
+      <c r="B83" t="n">
+        <v>4.320052563568</v>
+      </c>
+      <c r="C83" t="n">
+        <v>-3.999103954482208</v>
+      </c>
+      <c r="D83" t="n">
+        <v>-119.0640422865435</v>
+      </c>
+      <c r="E83" t="n">
+        <v>4.378151988783666</v>
+      </c>
+      <c r="F83" t="n">
+        <v>2.68742765562975</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="n">
+        <v>44927</v>
+      </c>
+      <c r="B84" t="n">
+        <v>5.712433228694</v>
+      </c>
+      <c r="C84" t="n">
+        <v>32.23064174885897</v>
+      </c>
+      <c r="D84" t="n">
+        <v>-755.9821478211799</v>
+      </c>
+      <c r="E84" t="n">
+        <v>4.844166181242</v>
+      </c>
+      <c r="F84" t="n">
+        <v>3.236032211899166</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="n">
+        <v>44958</v>
+      </c>
+      <c r="B85" t="n">
+        <v>6.045508733396</v>
+      </c>
+      <c r="C85" t="n">
+        <v>5.830711561387458</v>
+      </c>
+      <c r="D85" t="n">
+        <v>1424.985591891231</v>
+      </c>
+      <c r="E85" t="n">
+        <v>5.359331508552667</v>
+      </c>
+      <c r="F85" t="n">
+        <v>3.706788727378667</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="n">
+        <v>44986</v>
+      </c>
+      <c r="B86" t="n">
+        <v>5.591998385677</v>
+      </c>
+      <c r="C86" t="n">
+        <v>-7.501607684623179</v>
+      </c>
+      <c r="D86" t="n">
+        <v>403.5471459279038</v>
+      </c>
+      <c r="E86" t="n">
+        <v>5.783313449255666</v>
+      </c>
+      <c r="F86" t="n">
+        <v>4.080245149950417</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="n">
+        <v>45017</v>
+      </c>
+      <c r="B87" t="n">
+        <v>4.220350691848</v>
+      </c>
+      <c r="C87" t="n">
+        <v>-24.52875697071468</v>
+      </c>
+      <c r="D87" t="n">
+        <v>178.7747808725705</v>
+      </c>
+      <c r="E87" t="n">
+        <v>5.285952603640333</v>
+      </c>
+      <c r="F87" t="n">
+        <v>4.305783326855249</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="n">
+        <v>45047</v>
+      </c>
+      <c r="B88" t="n">
+        <v>4.003280784883</v>
+      </c>
+      <c r="C88" t="n">
+        <v>-5.143409228628581</v>
+      </c>
+      <c r="D88" t="n">
+        <v>55.39903190672207</v>
+      </c>
+      <c r="E88" t="n">
+        <v>4.605209954136</v>
+      </c>
+      <c r="F88" t="n">
+        <v>4.424712574789917</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>